<commit_message>
MAJ tarif via Power Automate
</commit_message>
<xml_diff>
--- a/data/TarifVinom_Master.xlsx
+++ b/data/TarifVinom_Master.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30502"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30516"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oliviermouton/Library/CloudStorage/OneDrive-Bibliothèquespartagées-VINOM/Vinom - Documents/TARIF VINOM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{A968D4B3-F538-6E4D-B999-D2E2C89C0321}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A5407BF-8587-4F2F-98FA-DF8E64959BE1}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{A968D4B3-F538-6E4D-B999-D2E2C89C0321}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1AD70A2F-A7B7-4D46-A1FE-D10AD18B7BBA}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="640" windowWidth="26580" windowHeight="12460" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22456,7 +22456,7 @@
         <v>75</v>
       </c>
       <c r="L363">
-        <v>5.65</v>
+        <v>6.1</v>
       </c>
       <c r="M363">
         <v>648</v>
@@ -31181,16 +31181,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="A31:L31"/>
-    <mergeCell ref="A32:L32"/>
-    <mergeCell ref="A33:L33"/>
-    <mergeCell ref="A34:L34"/>
-    <mergeCell ref="A25:L25"/>
-    <mergeCell ref="A26:L26"/>
-    <mergeCell ref="A27:L27"/>
-    <mergeCell ref="A28:L28"/>
-    <mergeCell ref="A29:L29"/>
-    <mergeCell ref="A30:L30"/>
     <mergeCell ref="A24:L24"/>
     <mergeCell ref="A13:L13"/>
     <mergeCell ref="A14:L14"/>
@@ -31203,6 +31193,16 @@
     <mergeCell ref="A21:L21"/>
     <mergeCell ref="A22:L22"/>
     <mergeCell ref="A23:L23"/>
+    <mergeCell ref="A31:L31"/>
+    <mergeCell ref="A32:L32"/>
+    <mergeCell ref="A33:L33"/>
+    <mergeCell ref="A34:L34"/>
+    <mergeCell ref="A25:L25"/>
+    <mergeCell ref="A26:L26"/>
+    <mergeCell ref="A27:L27"/>
+    <mergeCell ref="A28:L28"/>
+    <mergeCell ref="A29:L29"/>
+    <mergeCell ref="A30:L30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -52297,15 +52297,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="8b06e530-ed80-4ff0-be41-2806c2470479" xsi:nil="true"/>
@@ -52318,14 +52309,23 @@
 </p:properties>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7553FD30-6571-495C-A9F0-180AD16AA241}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C0FE2C01-6340-45D6-8526-0AB30AB8259E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2DE35E19-146F-4A5C-934B-8F843242C74E}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2DE35E19-146F-4A5C-934B-8F843242C74E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C0FE2C01-6340-45D6-8526-0AB30AB8259E}"/>
 </file>
</xml_diff>